<commit_message>
Draft Learn more content columns for Beginner biases
Add Usually Confused With, Noticing Cue, and Further Reading URL to the
Bias Library, and fill Tier 1 only so we can judge content quality before
building any Learn more UI.

Co-authored-by: andreeanesu <andreeanesu@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/second-thought/data/source/cognitive_bias_trainer.xlsx
+++ b/second-thought/data/source/cognitive_bias_trainer.xlsx
@@ -648,7 +648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H61"/>
+  <dimension ref="A1:K61"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="11" min="1" max="1"/>
@@ -701,6 +701,21 @@
           <t>Tier</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Usually Confused With</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Noticing Cue</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Further Reading URL</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="60" customHeight="1" s="12">
       <c r="A2" s="19" t="inlineStr">
@@ -741,6 +756,21 @@
       <c r="H2" s="11" t="n">
         <v>1</v>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Belief Perseverance, Choice-Supportive Bias</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Am I mostly collecting evidence that already agrees with me?</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Confirmation_bias</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="60" customHeight="1" s="12">
       <c r="A3" s="19" t="inlineStr">
@@ -781,6 +811,21 @@
       <c r="H3" s="11" t="n">
         <v>1</v>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Framing Effect</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Would I pick the same number if I had never seen the first figure?</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Anchoring_(cognitive_bias)</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="60" customHeight="1" s="12">
       <c r="A4" s="19" t="inlineStr">
@@ -821,6 +866,21 @@
       <c r="H4" s="11" t="n">
         <v>1</v>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Recency Bias, Representativeness Heuristic</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Is this easy to recall — or actually common?</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Availability_heuristic</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="60" customHeight="1" s="12">
       <c r="A5" s="19" t="inlineStr">
@@ -861,6 +921,21 @@
       <c r="H5" s="11" t="n">
         <v>1</v>
       </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Actor-Observer Bias, Hostile Attribution Bias</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Would I give myself the same excuse if I were in their situation?</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Fundamental_attribution_error</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="60" customHeight="1" s="12">
       <c r="A6" s="19" t="inlineStr">
@@ -901,6 +976,21 @@
       <c r="H6" s="11" t="n">
         <v>1</v>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Actor-Observer Bias, Egocentric Bias</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Am I claiming the wins and blaming the situation for the losses?</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Self-serving_bias</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="60" customHeight="1" s="12">
       <c r="A7" s="19" t="inlineStr">
@@ -941,6 +1031,21 @@
       <c r="H7" s="11" t="n">
         <v>1</v>
       </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Loss Aversion, Status Quo Bias, Endowment Effect</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>If I were deciding for the first time today, would I still continue?</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Sunk_cost#Loss_aversion_and_the_sunk_cost_fallacy</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="60" customHeight="1" s="12">
       <c r="A8" s="19" t="inlineStr">
@@ -981,6 +1086,21 @@
       <c r="H8" s="11" t="n">
         <v>1</v>
       </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Loss Aversion</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Am I weighting one bad moment more heavily than equally strong good ones?</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Negativity_bias</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="60" customHeight="1" s="12">
       <c r="A9" s="19" t="inlineStr">
@@ -1021,6 +1141,21 @@
       <c r="H9" s="11" t="n">
         <v>1</v>
       </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Horn Effect, Authority Bias</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Am I rating other traits higher just because I already like this person?</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Halo_effect</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="60" customHeight="1" s="12">
       <c r="A10" s="19" t="inlineStr">
@@ -1061,6 +1196,21 @@
       <c r="H10" s="11" t="n">
         <v>1</v>
       </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Halo Effect</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Am I assuming more negatives because of one bad impression?</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Horn_effect</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="60" customHeight="1" s="12">
       <c r="A11" s="19" t="inlineStr">
@@ -1101,6 +1251,21 @@
       <c r="H11" s="11" t="n">
         <v>1</v>
       </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Availability Heuristic</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Whose stories am I missing because they did not “make it”?</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Survivorship_bias</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="60" customHeight="1" s="12">
       <c r="A12" s="19" t="inlineStr">
@@ -1141,6 +1306,21 @@
       <c r="H12" s="11" t="n">
         <v>1</v>
       </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Overconfidence Effect</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Did I predict this beforehand — or does it only feel obvious now?</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Hindsight_bias</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="60" customHeight="1" s="12">
       <c r="A13" s="19" t="inlineStr">
@@ -1181,6 +1361,21 @@
       <c r="H13" s="11" t="n">
         <v>1</v>
       </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>In-group Bias, Naive Realism</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Have I checked whether people outside my circle actually agree?</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/False_consensus_effect</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="60" customHeight="1" s="12">
       <c r="A14" s="19" t="inlineStr">
@@ -1221,6 +1416,21 @@
       <c r="H14" s="11" t="n">
         <v>1</v>
       </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Out-group Homogeneity Bias, False Consensus Effect</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Would I judge this the same way if they were outside my group?</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/In-group_favoritism</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="60" customHeight="1" s="12">
       <c r="A15" s="19" t="inlineStr">
@@ -1261,6 +1471,21 @@
       <c r="H15" s="11" t="n">
         <v>1</v>
       </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>In-group Bias, Representativeness Heuristic</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Am I treating “them” as all alike while seeing variety in my own group?</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Out-group_homogeneity</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="60" customHeight="1" s="12">
       <c r="A16" s="19" t="inlineStr">
@@ -1301,6 +1526,21 @@
       <c r="H16" s="11" t="n">
         <v>1</v>
       </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Anchoring Bias, Loss Aversion</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Would my choice change if the same facts were worded differently?</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Framing_effect_(psychology)</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="60" customHeight="1" s="12">
       <c r="A17" s="19" t="inlineStr">
@@ -1341,6 +1581,21 @@
       <c r="H17" s="11" t="n">
         <v>1</v>
       </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Sunk Cost Fallacy, Endowment Effect, Negativity Bias</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Am I avoiding a loss harder than I would chase an equal gain?</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Loss_aversion</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="60" customHeight="1" s="12">
       <c r="A18" s="19" t="inlineStr">
@@ -1381,6 +1636,21 @@
       <c r="H18" s="11" t="n">
         <v>1</v>
       </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Overconfidence Effect, Planning Fallacy, Illusion of Control</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>What would a realistic base rate say about my odds?</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Optimism_bias</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="60" customHeight="1" s="12">
       <c r="A19" s="19" t="inlineStr">
@@ -1421,6 +1691,21 @@
       <c r="H19" s="11" t="n">
         <v>1</v>
       </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Sunk Cost Fallacy, Endowment Effect, Normalcy Bias</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Am I keeping this because it is better — or just because it is current?</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Status_quo_bias</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="60" customHeight="1" s="12">
       <c r="A20" s="19" t="inlineStr">
@@ -1461,6 +1746,21 @@
       <c r="H20" s="11" t="n">
         <v>1</v>
       </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Overconfidence Effect</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Have I tested my confidence against feedback from someone more experienced?</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Dunning%E2%80%93Kruger_effect</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="60" customHeight="1" s="12">
       <c r="A21" s="19" t="inlineStr">
@@ -1500,6 +1800,21 @@
       </c>
       <c r="H21" s="11" t="n">
         <v>1</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Halo Effect, Bandwagon Effect</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Am I trusting this because of the title — or because of the reasons?</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Authority_bias</t>
+        </is>
       </c>
     </row>
     <row r="22">

</xml_diff>

<commit_message>
Replace noticing cues with clearer-term definitions
Rename the Learn more draft field to “In clearer terms” and fill Tier 1
with fuller, precise definitions that add depth beyond the quiz reflect
prompts.

Co-authored-by: andreeanesu <andreeanesu@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/second-thought/data/source/cognitive_bias_trainer.xlsx
+++ b/second-thought/data/source/cognitive_bias_trainer.xlsx
@@ -701,17 +701,17 @@
           <t>Tier</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="11" t="inlineStr">
         <is>
           <t>Usually Confused With</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Noticing Cue</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
+      <c r="J1" s="11" t="inlineStr">
+        <is>
+          <t>In clearer terms</t>
+        </is>
+      </c>
+      <c r="K1" s="11" t="inlineStr">
         <is>
           <t>Further Reading URL</t>
         </is>
@@ -756,17 +756,17 @@
       <c r="H2" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="11" t="inlineStr">
         <is>
           <t>Belief Perseverance, Choice-Supportive Bias</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Am I mostly collecting evidence that already agrees with me?</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
+      <c r="J2" s="11" t="inlineStr">
+        <is>
+          <t>The tendency to seek, interpret, favour, and remember information that supports what we already believe, while giving less weight to information that challenges it.</t>
+        </is>
+      </c>
+      <c r="K2" s="11" t="inlineStr">
         <is>
           <t>https://en.wikipedia.org/wiki/Confirmation_bias</t>
         </is>
@@ -811,17 +811,17 @@
       <c r="H3" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="11" t="inlineStr">
         <is>
           <t>Framing Effect</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Would I pick the same number if I had never seen the first figure?</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
+      <c r="J3" s="11" t="inlineStr">
+        <is>
+          <t>The tendency to rely too heavily on an initial piece of information (an “anchor”) when making estimates or decisions, even when that starting point is arbitrary.</t>
+        </is>
+      </c>
+      <c r="K3" s="11" t="inlineStr">
         <is>
           <t>https://en.wikipedia.org/wiki/Anchoring_(cognitive_bias)</t>
         </is>
@@ -866,17 +866,17 @@
       <c r="H4" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="11" t="inlineStr">
         <is>
           <t>Recency Bias, Representativeness Heuristic</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Is this easy to recall — or actually common?</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
+      <c r="J4" s="11" t="inlineStr">
+        <is>
+          <t>A mental shortcut where we judge how common or likely something is by how easily examples come to mind, which can make vivid or recent events feel more frequent than they are.</t>
+        </is>
+      </c>
+      <c r="K4" s="11" t="inlineStr">
         <is>
           <t>https://en.wikipedia.org/wiki/Availability_heuristic</t>
         </is>
@@ -921,17 +921,17 @@
       <c r="H5" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" s="11" t="inlineStr">
         <is>
           <t>Actor-Observer Bias, Hostile Attribution Bias</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Would I give myself the same excuse if I were in their situation?</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
+      <c r="J5" s="11" t="inlineStr">
+        <is>
+          <t>The tendency to explain other people’s actions mainly by their character or personality, while underestimating the role of the situation they are in.</t>
+        </is>
+      </c>
+      <c r="K5" s="11" t="inlineStr">
         <is>
           <t>https://en.wikipedia.org/wiki/Fundamental_attribution_error</t>
         </is>
@@ -976,17 +976,17 @@
       <c r="H6" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I6" s="11" t="inlineStr">
         <is>
           <t>Actor-Observer Bias, Egocentric Bias</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Am I claiming the wins and blaming the situation for the losses?</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
+      <c r="J6" s="11" t="inlineStr">
+        <is>
+          <t>The tendency to credit our successes to our own ability or effort, and to blame our failures on outside circumstances, bad luck, or other people.</t>
+        </is>
+      </c>
+      <c r="K6" s="11" t="inlineStr">
         <is>
           <t>https://en.wikipedia.org/wiki/Self-serving_bias</t>
         </is>
@@ -1031,17 +1031,17 @@
       <c r="H7" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I7" s="11" t="inlineStr">
         <is>
           <t>Loss Aversion, Status Quo Bias, Endowment Effect</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>If I were deciding for the first time today, would I still continue?</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
+      <c r="J7" s="11" t="inlineStr">
+        <is>
+          <t>The tendency to continue with a plan or investment because of what we have already put in (time, money, or effort), rather than because future benefits still justify it.</t>
+        </is>
+      </c>
+      <c r="K7" s="11" t="inlineStr">
         <is>
           <t>https://en.wikipedia.org/wiki/Sunk_cost#Loss_aversion_and_the_sunk_cost_fallacy</t>
         </is>
@@ -1086,17 +1086,17 @@
       <c r="H8" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I8" s="11" t="inlineStr">
         <is>
           <t>Loss Aversion</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Am I weighting one bad moment more heavily than equally strong good ones?</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
+      <c r="J8" s="11" t="inlineStr">
+        <is>
+          <t>The tendency for negative events, information, or emotions to affect us more strongly than positive ones of equal intensity.</t>
+        </is>
+      </c>
+      <c r="K8" s="11" t="inlineStr">
         <is>
           <t>https://en.wikipedia.org/wiki/Negativity_bias</t>
         </is>
@@ -1141,17 +1141,17 @@
       <c r="H9" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I9" s="11" t="inlineStr">
         <is>
           <t>Horn Effect, Authority Bias</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>Am I rating other traits higher just because I already like this person?</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
+      <c r="J9" s="11" t="inlineStr">
+        <is>
+          <t>When a positive overall impression of someone (or something) spills over and makes us rate their other traits more favourably than the evidence supports.</t>
+        </is>
+      </c>
+      <c r="K9" s="11" t="inlineStr">
         <is>
           <t>https://en.wikipedia.org/wiki/Halo_effect</t>
         </is>
@@ -1196,17 +1196,17 @@
       <c r="H10" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I10" s="11" t="inlineStr">
         <is>
           <t>Halo Effect</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>Am I assuming more negatives because of one bad impression?</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
+      <c r="J10" s="11" t="inlineStr">
+        <is>
+          <t>When a negative overall impression of someone (or something) spills over and makes us rate their other traits more harshly than the evidence supports.</t>
+        </is>
+      </c>
+      <c r="K10" s="11" t="inlineStr">
         <is>
           <t>https://en.wikipedia.org/wiki/Horn_effect</t>
         </is>
@@ -1251,17 +1251,17 @@
       <c r="H11" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I11" s="11" t="inlineStr">
         <is>
           <t>Availability Heuristic</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>Whose stories am I missing because they did not “make it”?</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
+      <c r="J11" s="11" t="inlineStr">
+        <is>
+          <t>The tendency to draw conclusions from the people or cases that “made it,” while overlooking those that failed, dropped out, or were never visible — which can distort what we think works.</t>
+        </is>
+      </c>
+      <c r="K11" s="11" t="inlineStr">
         <is>
           <t>https://en.wikipedia.org/wiki/Survivorship_bias</t>
         </is>
@@ -1306,17 +1306,17 @@
       <c r="H12" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>Overconfidence Effect</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>Did I predict this beforehand — or does it only feel obvious now?</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
+      <c r="J12" s="11" t="inlineStr">
+        <is>
+          <t>The tendency, after an outcome is known, to see it as more predictable than it really was, and to believe we “knew it all along.”</t>
+        </is>
+      </c>
+      <c r="K12" s="11" t="inlineStr">
         <is>
           <t>https://en.wikipedia.org/wiki/Hindsight_bias</t>
         </is>
@@ -1361,17 +1361,17 @@
       <c r="H13" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I13" s="11" t="inlineStr">
         <is>
           <t>In-group Bias, Naive Realism</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>Have I checked whether people outside my circle actually agree?</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
+      <c r="J13" s="11" t="inlineStr">
+        <is>
+          <t>The tendency to overestimate how widely others share our beliefs, preferences, and behaviours.</t>
+        </is>
+      </c>
+      <c r="K13" s="11" t="inlineStr">
         <is>
           <t>https://en.wikipedia.org/wiki/False_consensus_effect</t>
         </is>
@@ -1416,17 +1416,17 @@
       <c r="H14" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I14" s="11" t="inlineStr">
         <is>
           <t>Out-group Homogeneity Bias, False Consensus Effect</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>Would I judge this the same way if they were outside my group?</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
+      <c r="J14" s="11" t="inlineStr">
+        <is>
+          <t>The tendency to favour people who belong to our own group — giving them more trust, warmth, or benefit of the doubt than we give outsiders.</t>
+        </is>
+      </c>
+      <c r="K14" s="11" t="inlineStr">
         <is>
           <t>https://en.wikipedia.org/wiki/In-group_favoritism</t>
         </is>
@@ -1471,17 +1471,17 @@
       <c r="H15" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="I15" s="11" t="inlineStr">
         <is>
           <t>In-group Bias, Representativeness Heuristic</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>Am I treating “them” as all alike while seeing variety in my own group?</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
+      <c r="J15" s="11" t="inlineStr">
+        <is>
+          <t>The tendency to see people in other groups as more alike than they are, while seeing members of our own group as more varied and individual.</t>
+        </is>
+      </c>
+      <c r="K15" s="11" t="inlineStr">
         <is>
           <t>https://en.wikipedia.org/wiki/Out-group_homogeneity</t>
         </is>
@@ -1526,17 +1526,17 @@
       <c r="H16" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="I16" s="11" t="inlineStr">
         <is>
           <t>Anchoring Bias, Loss Aversion</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>Would my choice change if the same facts were worded differently?</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
+      <c r="J16" s="11" t="inlineStr">
+        <is>
+          <t>The tendency for the same facts to lead to different choices depending on how they are worded or presented — for example as gains versus losses.</t>
+        </is>
+      </c>
+      <c r="K16" s="11" t="inlineStr">
         <is>
           <t>https://en.wikipedia.org/wiki/Framing_effect_(psychology)</t>
         </is>
@@ -1581,17 +1581,17 @@
       <c r="H17" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I17" s="11" t="inlineStr">
         <is>
           <t>Sunk Cost Fallacy, Endowment Effect, Negativity Bias</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>Am I avoiding a loss harder than I would chase an equal gain?</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
+      <c r="J17" s="11" t="inlineStr">
+        <is>
+          <t>The tendency for losses to feel more painful than gains of the same size feel rewarding, which can make us overly cautious about potential losses.</t>
+        </is>
+      </c>
+      <c r="K17" s="11" t="inlineStr">
         <is>
           <t>https://en.wikipedia.org/wiki/Loss_aversion</t>
         </is>
@@ -1636,17 +1636,17 @@
       <c r="H18" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="I18" s="11" t="inlineStr">
         <is>
           <t>Overconfidence Effect, Planning Fallacy, Illusion of Control</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>What would a realistic base rate say about my odds?</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
+      <c r="J18" s="11" t="inlineStr">
+        <is>
+          <t>The tendency to overestimate how likely good things are to happen to us, and to underestimate our personal risk of bad outcomes compared with other people.</t>
+        </is>
+      </c>
+      <c r="K18" s="11" t="inlineStr">
         <is>
           <t>https://en.wikipedia.org/wiki/Optimism_bias</t>
         </is>
@@ -1691,17 +1691,17 @@
       <c r="H19" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I19" s="11" t="inlineStr">
         <is>
           <t>Sunk Cost Fallacy, Endowment Effect, Normalcy Bias</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>Am I keeping this because it is better — or just because it is current?</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
+      <c r="J19" s="11" t="inlineStr">
+        <is>
+          <t>The tendency to prefer the current state of affairs and to treat “keeping things as they are” as the default choice, even when change might be better.</t>
+        </is>
+      </c>
+      <c r="K19" s="11" t="inlineStr">
         <is>
           <t>https://en.wikipedia.org/wiki/Status_quo_bias</t>
         </is>
@@ -1746,17 +1746,17 @@
       <c r="H20" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="I20" s="11" t="inlineStr">
         <is>
           <t>Overconfidence Effect</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>Have I tested my confidence against feedback from someone more experienced?</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
+      <c r="J20" s="11" t="inlineStr">
+        <is>
+          <t>A pattern where people with limited skill or knowledge in an area overestimate how competent they are, partly because the same gaps that cause mistakes also hide those mistakes from view.</t>
+        </is>
+      </c>
+      <c r="K20" s="11" t="inlineStr">
         <is>
           <t>https://en.wikipedia.org/wiki/Dunning%E2%80%93Kruger_effect</t>
         </is>
@@ -1801,17 +1801,17 @@
       <c r="H21" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="I21" s="11" t="inlineStr">
         <is>
           <t>Halo Effect, Bandwagon Effect</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>Am I trusting this because of the title — or because of the reasons?</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
+      <c r="J21" s="11" t="inlineStr">
+        <is>
+          <t>The tendency to trust or follow the views of someone seen as an authority more than the strength of their arguments alone would justify.</t>
+        </is>
+      </c>
+      <c r="K21" s="11" t="inlineStr">
         <is>
           <t>https://en.wikipedia.org/wiki/Authority_bias</t>
         </is>

</xml_diff>

<commit_message>
Expand Learn more draft definitions across all 60 biases
Use Definition as the Learn more label, fill fuller definitions plus
confused-with pairs and Wikipedia links for every bias, and sync JSON
via the Excel converter.

Co-authored-by: andreeanesu <andreeanesu@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/second-thought/data/source/cognitive_bias_trainer.xlsx
+++ b/second-thought/data/source/cognitive_bias_trainer.xlsx
@@ -648,7 +648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K61"/>
+  <dimension ref="A1:J61"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="11" min="1" max="1"/>
@@ -708,11 +708,6 @@
       </c>
       <c r="J1" s="11" t="inlineStr">
         <is>
-          <t>In clearer terms</t>
-        </is>
-      </c>
-      <c r="K1" s="11" t="inlineStr">
-        <is>
           <t>Further Reading URL</t>
         </is>
       </c>
@@ -730,7 +725,7 @@
       </c>
       <c r="C2" s="19" t="inlineStr">
         <is>
-          <t>We tend to search for, interpret, and recall information that confirms our existing beliefs.</t>
+          <t>The tendency to seek, interpret, favour, and remember information that supports what we already believe, while giving less weight to information that challenges it.</t>
         </is>
       </c>
       <c r="D2" s="19" t="inlineStr">
@@ -763,11 +758,6 @@
       </c>
       <c r="J2" s="11" t="inlineStr">
         <is>
-          <t>The tendency to seek, interpret, favour, and remember information that supports what we already believe, while giving less weight to information that challenges it.</t>
-        </is>
-      </c>
-      <c r="K2" s="11" t="inlineStr">
-        <is>
           <t>https://en.wikipedia.org/wiki/Confirmation_bias</t>
         </is>
       </c>
@@ -785,7 +775,7 @@
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
-          <t>We rely too heavily on the first piece of information offered (the 'anchor') when making decisions.</t>
+          <t>The tendency to rely too heavily on an initial piece of information (an “anchor”) when making estimates or decisions, even when that starting point is arbitrary.</t>
         </is>
       </c>
       <c r="D3" s="19" t="inlineStr">
@@ -818,11 +808,6 @@
       </c>
       <c r="J3" s="11" t="inlineStr">
         <is>
-          <t>The tendency to rely too heavily on an initial piece of information (an “anchor”) when making estimates or decisions, even when that starting point is arbitrary.</t>
-        </is>
-      </c>
-      <c r="K3" s="11" t="inlineStr">
-        <is>
           <t>https://en.wikipedia.org/wiki/Anchoring_(cognitive_bias)</t>
         </is>
       </c>
@@ -840,7 +825,7 @@
       </c>
       <c r="C4" s="19" t="inlineStr">
         <is>
-          <t>We judge the likelihood of events based on how easily examples come to mind.</t>
+          <t>A mental shortcut where we judge how common or likely something is by how easily examples come to mind, which can make vivid or recent events feel more frequent than they are.</t>
         </is>
       </c>
       <c r="D4" s="19" t="inlineStr">
@@ -873,11 +858,6 @@
       </c>
       <c r="J4" s="11" t="inlineStr">
         <is>
-          <t>A mental shortcut where we judge how common or likely something is by how easily examples come to mind, which can make vivid or recent events feel more frequent than they are.</t>
-        </is>
-      </c>
-      <c r="K4" s="11" t="inlineStr">
-        <is>
           <t>https://en.wikipedia.org/wiki/Availability_heuristic</t>
         </is>
       </c>
@@ -895,7 +875,7 @@
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>We judge others' behavior as caused by their character, while excusing our own behavior as caused by circumstances.</t>
+          <t>The tendency to explain other people’s actions mainly by their character or personality, while underestimating the role of the situation they are in.</t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
@@ -928,11 +908,6 @@
       </c>
       <c r="J5" s="11" t="inlineStr">
         <is>
-          <t>The tendency to explain other people’s actions mainly by their character or personality, while underestimating the role of the situation they are in.</t>
-        </is>
-      </c>
-      <c r="K5" s="11" t="inlineStr">
-        <is>
           <t>https://en.wikipedia.org/wiki/Fundamental_attribution_error</t>
         </is>
       </c>
@@ -950,7 +925,7 @@
       </c>
       <c r="C6" s="19" t="inlineStr">
         <is>
-          <t>We attribute our successes to our own abilities and our failures to external circumstances.</t>
+          <t>The tendency to credit our successes to our own ability or effort, and to blame our failures on outside circumstances, bad luck, or other people.</t>
         </is>
       </c>
       <c r="D6" s="19" t="inlineStr">
@@ -983,11 +958,6 @@
       </c>
       <c r="J6" s="11" t="inlineStr">
         <is>
-          <t>The tendency to credit our successes to our own ability or effort, and to blame our failures on outside circumstances, bad luck, or other people.</t>
-        </is>
-      </c>
-      <c r="K6" s="11" t="inlineStr">
-        <is>
           <t>https://en.wikipedia.org/wiki/Self-serving_bias</t>
         </is>
       </c>
@@ -1005,7 +975,7 @@
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>We continue investing in something because of what we've already invested, rather than evaluating future value.</t>
+          <t>The tendency to continue with a plan or investment because of what we have already put in (time, money, or effort), rather than because future benefits still justify it.</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
@@ -1038,11 +1008,6 @@
       </c>
       <c r="J7" s="11" t="inlineStr">
         <is>
-          <t>The tendency to continue with a plan or investment because of what we have already put in (time, money, or effort), rather than because future benefits still justify it.</t>
-        </is>
-      </c>
-      <c r="K7" s="11" t="inlineStr">
-        <is>
           <t>https://en.wikipedia.org/wiki/Sunk_cost#Loss_aversion_and_the_sunk_cost_fallacy</t>
         </is>
       </c>
@@ -1060,7 +1025,7 @@
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
-          <t>We give more psychological weight to negative experiences than to positive ones of equal intensity.</t>
+          <t>The tendency for negative events, information, or emotions to affect us more strongly than positive ones of equal intensity.</t>
         </is>
       </c>
       <c r="D8" s="19" t="inlineStr">
@@ -1093,11 +1058,6 @@
       </c>
       <c r="J8" s="11" t="inlineStr">
         <is>
-          <t>The tendency for negative events, information, or emotions to affect us more strongly than positive ones of equal intensity.</t>
-        </is>
-      </c>
-      <c r="K8" s="11" t="inlineStr">
-        <is>
           <t>https://en.wikipedia.org/wiki/Negativity_bias</t>
         </is>
       </c>
@@ -1115,7 +1075,7 @@
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>Our overall impression of a person influences how we judge their specific traits, so one positive trait makes us assume other positive traits.</t>
+          <t>When a positive overall impression of someone (or something) spills over and makes us rate their other traits more favourably than the evidence supports.</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
@@ -1148,11 +1108,6 @@
       </c>
       <c r="J9" s="11" t="inlineStr">
         <is>
-          <t>When a positive overall impression of someone (or something) spills over and makes us rate their other traits more favourably than the evidence supports.</t>
-        </is>
-      </c>
-      <c r="K9" s="11" t="inlineStr">
-        <is>
           <t>https://en.wikipedia.org/wiki/Halo_effect</t>
         </is>
       </c>
@@ -1170,7 +1125,7 @@
       </c>
       <c r="C10" s="19" t="inlineStr">
         <is>
-          <t>One negative trait about a person leads us to assume other negative traits, the opposite of the halo effect.</t>
+          <t>When a negative overall impression of someone (or something) spills over and makes us rate their other traits more harshly than the evidence supports.</t>
         </is>
       </c>
       <c r="D10" s="19" t="inlineStr">
@@ -1203,11 +1158,6 @@
       </c>
       <c r="J10" s="11" t="inlineStr">
         <is>
-          <t>When a negative overall impression of someone (or something) spills over and makes us rate their other traits more harshly than the evidence supports.</t>
-        </is>
-      </c>
-      <c r="K10" s="11" t="inlineStr">
-        <is>
           <t>https://en.wikipedia.org/wiki/Horn_effect</t>
         </is>
       </c>
@@ -1225,7 +1175,7 @@
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>We focus on the people or things that 'survived' a process, while overlooking those that didn't, skewing our conclusions.</t>
+          <t>The tendency to draw conclusions from the people or cases that “made it,” while overlooking those that failed, dropped out, or were never visible — which can distort what we think works.</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
@@ -1258,11 +1208,6 @@
       </c>
       <c r="J11" s="11" t="inlineStr">
         <is>
-          <t>The tendency to draw conclusions from the people or cases that “made it,” while overlooking those that failed, dropped out, or were never visible — which can distort what we think works.</t>
-        </is>
-      </c>
-      <c r="K11" s="11" t="inlineStr">
-        <is>
           <t>https://en.wikipedia.org/wiki/Survivorship_bias</t>
         </is>
       </c>
@@ -1280,7 +1225,7 @@
       </c>
       <c r="C12" s="19" t="inlineStr">
         <is>
-          <t>After an event happens, we tend to believe we 'knew it all along,' even if we couldn't have predicted it beforehand.</t>
+          <t>The tendency, after an outcome is known, to see it as more predictable than it really was, and to believe we “knew it all along.”</t>
         </is>
       </c>
       <c r="D12" s="19" t="inlineStr">
@@ -1313,11 +1258,6 @@
       </c>
       <c r="J12" s="11" t="inlineStr">
         <is>
-          <t>The tendency, after an outcome is known, to see it as more predictable than it really was, and to believe we “knew it all along.”</t>
-        </is>
-      </c>
-      <c r="K12" s="11" t="inlineStr">
-        <is>
           <t>https://en.wikipedia.org/wiki/Hindsight_bias</t>
         </is>
       </c>
@@ -1335,7 +1275,7 @@
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>We overestimate how much other people share our beliefs, opinions, and behaviors.</t>
+          <t>The tendency to overestimate how widely others share our beliefs, preferences, and behaviours.</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -1368,11 +1308,6 @@
       </c>
       <c r="J13" s="11" t="inlineStr">
         <is>
-          <t>The tendency to overestimate how widely others share our beliefs, preferences, and behaviours.</t>
-        </is>
-      </c>
-      <c r="K13" s="11" t="inlineStr">
-        <is>
           <t>https://en.wikipedia.org/wiki/False_consensus_effect</t>
         </is>
       </c>
@@ -1390,7 +1325,7 @@
       </c>
       <c r="C14" s="19" t="inlineStr">
         <is>
-          <t>We favor members of our own group over members of other groups, often unconsciously.</t>
+          <t>The tendency to favour people who belong to our own group — giving them more trust, warmth, or benefit of the doubt than we give outsiders.</t>
         </is>
       </c>
       <c r="D14" s="19" t="inlineStr">
@@ -1423,11 +1358,6 @@
       </c>
       <c r="J14" s="11" t="inlineStr">
         <is>
-          <t>The tendency to favour people who belong to our own group — giving them more trust, warmth, or benefit of the doubt than we give outsiders.</t>
-        </is>
-      </c>
-      <c r="K14" s="11" t="inlineStr">
-        <is>
           <t>https://en.wikipedia.org/wiki/In-group_favoritism</t>
         </is>
       </c>
@@ -1445,7 +1375,7 @@
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>We tend to see members of other groups as more similar to each other than they really are, while seeing our own group as diverse.</t>
+          <t>The tendency to see people in other groups as more alike than they are, while seeing members of our own group as more varied and individual.</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -1478,11 +1408,6 @@
       </c>
       <c r="J15" s="11" t="inlineStr">
         <is>
-          <t>The tendency to see people in other groups as more alike than they are, while seeing members of our own group as more varied and individual.</t>
-        </is>
-      </c>
-      <c r="K15" s="11" t="inlineStr">
-        <is>
           <t>https://en.wikipedia.org/wiki/Out-group_homogeneity</t>
         </is>
       </c>
@@ -1500,7 +1425,7 @@
       </c>
       <c r="C16" s="19" t="inlineStr">
         <is>
-          <t>Our decisions are influenced by how information is presented (framed), even when the underlying facts are the same.</t>
+          <t>The tendency for the same facts to lead to different choices depending on how they are worded or presented — for example as gains versus losses.</t>
         </is>
       </c>
       <c r="D16" s="19" t="inlineStr">
@@ -1533,11 +1458,6 @@
       </c>
       <c r="J16" s="11" t="inlineStr">
         <is>
-          <t>The tendency for the same facts to lead to different choices depending on how they are worded or presented — for example as gains versus losses.</t>
-        </is>
-      </c>
-      <c r="K16" s="11" t="inlineStr">
-        <is>
           <t>https://en.wikipedia.org/wiki/Framing_effect_(psychology)</t>
         </is>
       </c>
@@ -1555,7 +1475,7 @@
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>The pain of losing something feels psychologically stronger than the pleasure of gaining something of equal value.</t>
+          <t>The tendency for losses to feel more painful than gains of the same size feel rewarding, which can make us overly cautious about potential losses.</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1588,11 +1508,6 @@
       </c>
       <c r="J17" s="11" t="inlineStr">
         <is>
-          <t>The tendency for losses to feel more painful than gains of the same size feel rewarding, which can make us overly cautious about potential losses.</t>
-        </is>
-      </c>
-      <c r="K17" s="11" t="inlineStr">
-        <is>
           <t>https://en.wikipedia.org/wiki/Loss_aversion</t>
         </is>
       </c>
@@ -1610,7 +1525,7 @@
       </c>
       <c r="C18" s="19" t="inlineStr">
         <is>
-          <t>We tend to overestimate the likelihood of positive events happening to us and underestimate the likelihood of negative ones.</t>
+          <t>The tendency to overestimate how likely good things are to happen to us, and to underestimate our personal risk of bad outcomes compared with other people.</t>
         </is>
       </c>
       <c r="D18" s="19" t="inlineStr">
@@ -1643,11 +1558,6 @@
       </c>
       <c r="J18" s="11" t="inlineStr">
         <is>
-          <t>The tendency to overestimate how likely good things are to happen to us, and to underestimate our personal risk of bad outcomes compared with other people.</t>
-        </is>
-      </c>
-      <c r="K18" s="11" t="inlineStr">
-        <is>
           <t>https://en.wikipedia.org/wiki/Optimism_bias</t>
         </is>
       </c>
@@ -1665,7 +1575,7 @@
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>We prefer things to stay the same, and treat the current state as a reasonable default, even when change might be better.</t>
+          <t>The tendency to prefer the current state of affairs and to treat “keeping things as they are” as the default choice, even when change might be better.</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -1698,11 +1608,6 @@
       </c>
       <c r="J19" s="11" t="inlineStr">
         <is>
-          <t>The tendency to prefer the current state of affairs and to treat “keeping things as they are” as the default choice, even when change might be better.</t>
-        </is>
-      </c>
-      <c r="K19" s="11" t="inlineStr">
-        <is>
           <t>https://en.wikipedia.org/wiki/Status_quo_bias</t>
         </is>
       </c>
@@ -1720,7 +1625,7 @@
       </c>
       <c r="C20" s="19" t="inlineStr">
         <is>
-          <t>People with limited knowledge or skill in an area tend to overestimate their own competence.</t>
+          <t>A pattern where people with limited skill or knowledge in an area overestimate how competent they are, partly because the same gaps that cause mistakes also hide those mistakes from view.</t>
         </is>
       </c>
       <c r="D20" s="19" t="inlineStr">
@@ -1753,11 +1658,6 @@
       </c>
       <c r="J20" s="11" t="inlineStr">
         <is>
-          <t>A pattern where people with limited skill or knowledge in an area overestimate how competent they are, partly because the same gaps that cause mistakes also hide those mistakes from view.</t>
-        </is>
-      </c>
-      <c r="K20" s="11" t="inlineStr">
-        <is>
           <t>https://en.wikipedia.org/wiki/Dunning%E2%80%93Kruger_effect</t>
         </is>
       </c>
@@ -1775,7 +1675,7 @@
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>We tend to attribute greater accuracy and trust to the opinions of an authority figure, regardless of the actual content.</t>
+          <t>The tendency to trust or follow the views of someone seen as an authority more than the strength of their arguments alone would justify.</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -1808,11 +1708,6 @@
       </c>
       <c r="J21" s="11" t="inlineStr">
         <is>
-          <t>The tendency to trust or follow the views of someone seen as an authority more than the strength of their arguments alone would justify.</t>
-        </is>
-      </c>
-      <c r="K21" s="11" t="inlineStr">
-        <is>
           <t>https://en.wikipedia.org/wiki/Authority_bias</t>
         </is>
       </c>
@@ -1830,7 +1725,7 @@
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>We routinely underestimate how long tasks will take and overestimate how smoothly they will go.</t>
+          <t>The tendency to underestimate how long a task will take and how many obstacles will appear, even when similar tasks have overrun before.</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -1856,6 +1751,16 @@
       <c r="H22" s="11" t="n">
         <v>2</v>
       </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Optimism Bias, Overconfidence Effect</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Planning_fallacy</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
@@ -1870,7 +1775,7 @@
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>We give more weight to recent events than to older ones, even when the older pattern matters more.</t>
+          <t>The tendency to give recent information more weight than older information, even when the longer track record is more informative.</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr">
@@ -1896,6 +1801,16 @@
       <c r="H23" s="11" t="n">
         <v>2</v>
       </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Availability Heuristic</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Recency_bias</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
@@ -1910,7 +1825,7 @@
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>We are more likely to adopt a belief or behaviour because many others are doing it.</t>
+          <t>The tendency to adopt a belief or behaviour because many other people are doing so, treating popularity as a signal that it must be right.</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -1936,6 +1851,16 @@
       <c r="H24" s="11" t="n">
         <v>2</v>
       </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Authority Bias, In-group Bias</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Bandwagon_effect</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
@@ -1950,7 +1875,7 @@
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>We tend to like things more simply because we have encountered them before.</t>
+          <t>The tendency to like people, ideas, or things more simply because we have encountered them before, even without stronger reasons to prefer them.</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
@@ -1976,6 +1901,16 @@
       <c r="H25" s="11" t="n">
         <v>2</v>
       </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Status Quo Bias, Illusory Truth Effect</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Mere-exposure_effect</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
@@ -1990,7 +1925,7 @@
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>We value things more highly simply because we already own them.</t>
+          <t>The tendency to value something more highly once we own it than we would if the same item belonged to someone else.</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2016,6 +1951,16 @@
       <c r="H26" s="11" t="n">
         <v>2</v>
       </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Loss Aversion, Status Quo Bias, Sunk Cost Fallacy</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Endowment_effect</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
@@ -2030,7 +1975,7 @@
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>We expect random events to balance out in the short run, as if past outcomes change future odds.</t>
+          <t>The belief that a random event is “due” after a streak of opposite outcomes, as if chance keeps a short-run balance sheet.</t>
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr">
@@ -2056,6 +2001,16 @@
       <c r="H27" s="11" t="n">
         <v>2</v>
       </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Clustering Illusion, Illusion of Control</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Gambler%27s_fallacy</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
@@ -2070,7 +2025,7 @@
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>We see meaningful patterns in small sets of random or unrelated events.</t>
+          <t>The tendency to see meaningful patterns or streaks in small samples of random or unrelated events.</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -2096,6 +2051,16 @@
       <c r="H28" s="11" t="n">
         <v>2</v>
       </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Gambler's Fallacy, Illusory Correlation</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Clustering_illusion</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="11" t="inlineStr">
@@ -2110,7 +2075,7 @@
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>We judge how likely something is by how much it resembles a stereotype, instead of using actual odds.</t>
+          <t>A mental shortcut where we judge probability by how much something resembles a familiar stereotype or story, instead of using actual base rates.</t>
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr">
@@ -2136,6 +2101,16 @@
       <c r="H29" s="11" t="n">
         <v>2</v>
       </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Base Rate Neglect, Availability Heuristic</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Representativeness_heuristic</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
@@ -2150,7 +2125,7 @@
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>We ignore general base-rate information and focus on specific, vivid details instead.</t>
+          <t>The tendency to ignore general statistical information about how common something is, and to focus instead on specific, vivid details.</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -2176,6 +2151,16 @@
       <c r="H30" s="11" t="n">
         <v>2</v>
       </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Representativeness Heuristic, Availability Heuristic</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Base_rate_fallacy</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
@@ -2190,7 +2175,7 @@
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>We judge an experience mainly by its most intense moment and how it ended, not the whole duration.</t>
+          <t>The tendency to judge an experience mainly by its most intense moment and how it ended, rather than by the whole duration.</t>
         </is>
       </c>
       <c r="D31" s="11" t="inlineStr">
@@ -2216,6 +2201,16 @@
       <c r="H31" s="11" t="n">
         <v>2</v>
       </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Negativity Bias</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Peak%E2%80%93end_rule</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
@@ -2230,7 +2225,7 @@
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>After making a choice, we remember the chosen option more favourably and downplay its downsides.</t>
+          <t>The tendency, after we have chosen an option, to remember it more favourably and to downplay its downsides or the appeal of alternatives.</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
@@ -2256,6 +2251,16 @@
       <c r="H32" s="11" t="n">
         <v>2</v>
       </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Confirmation Bias, Cognitive Dissonance</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Choice-supportive_bias</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="11" t="inlineStr">
@@ -2270,7 +2275,7 @@
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>We overestimate how much influence we have over outcomes that are mostly chance or outside our control.</t>
+          <t>The tendency to overestimate how much influence our actions have over outcomes that are largely random or outside our control.</t>
         </is>
       </c>
       <c r="D33" s="11" t="inlineStr">
@@ -2296,6 +2301,16 @@
       <c r="H33" s="11" t="n">
         <v>2</v>
       </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Optimism Bias, Gambler's Fallacy</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Illusion_of_control</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
@@ -2310,7 +2325,7 @@
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>We overestimate how much other people notice our appearance, mistakes, or behaviour.</t>
+          <t>The tendency to overestimate how much other people notice our appearance, mistakes, or behaviour.</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2336,6 +2351,16 @@
       <c r="H34" s="11" t="n">
         <v>2</v>
       </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Illusion of Transparency, Egocentric Bias</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Spotlight_effect</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="11" t="inlineStr">
@@ -2350,7 +2375,7 @@
       </c>
       <c r="C35" s="11" t="inlineStr">
         <is>
-          <t>When our actions clash with our beliefs, we often change our beliefs or excuses rather than face the clash.</t>
+          <t>The mental discomfort that arises when our actions conflict with our beliefs, often leading us to justify, minimise, or reframe what we did.</t>
         </is>
       </c>
       <c r="D35" s="11" t="inlineStr">
@@ -2376,6 +2401,16 @@
       <c r="H35" s="11" t="n">
         <v>2</v>
       </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Choice-Supportive Bias, Belief Perseverance</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Cognitive_dissonance</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="11" t="inlineStr">
@@ -2390,7 +2425,7 @@
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>We keep believing something even after the evidence supporting it has been weakened or removed.</t>
+          <t>The tendency to hold on to a belief even after the evidence that supported it has been weakened or removed.</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -2416,6 +2451,16 @@
       <c r="H36" s="11" t="n">
         <v>2</v>
       </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Confirmation Bias, Semmelweis Reflex</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Belief_perseverance</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="11" t="inlineStr">
@@ -2430,7 +2475,7 @@
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>We underestimate the chance of disruption and assume things will keep going as they usually do.</t>
+          <t>The tendency to underestimate the likelihood of serious disruption and to assume that life will continue in the usual way.</t>
         </is>
       </c>
       <c r="D37" s="11" t="inlineStr">
@@ -2456,6 +2501,16 @@
       <c r="H37" s="11" t="n">
         <v>2</v>
       </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Status Quo Bias, Optimism Bias</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Normalcy_bias</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="11" t="inlineStr">
@@ -2470,7 +2525,7 @@
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Once we know something, we find it hard to imagine not knowing it.</t>
+          <t>The difficulty of remembering what it was like not to know something, which can make experts skip steps that beginners still need.</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -2496,6 +2551,16 @@
       <c r="H38" s="11" t="n">
         <v>2</v>
       </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>False Consensus Effect, Egocentric Bias</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Curse_of_knowledge</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="11" t="inlineStr">
@@ -2510,7 +2575,7 @@
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>We perceive a link between two things when none exists, or see a stronger link than the data supports.</t>
+          <t>The tendency to perceive a relationship between two things when none exists, or to see a stronger link than the evidence supports.</t>
         </is>
       </c>
       <c r="D39" s="11" t="inlineStr">
@@ -2536,6 +2601,16 @@
       <c r="H39" s="11" t="n">
         <v>2</v>
       </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Clustering Illusion, Confirmation Bias</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Illusory_correlation</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="11" t="inlineStr">
@@ -2550,7 +2625,7 @@
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>We judge a detailed, specific story as more likely than a broader, more general one.</t>
+          <t>The tendency to judge a detailed, specific scenario as more probable than a broader one, even though added detail usually makes an event less likely.</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -2576,6 +2651,16 @@
       <c r="H40" s="11" t="n">
         <v>2</v>
       </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Representativeness Heuristic</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Conjunction_fallacy</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="11" t="inlineStr">
@@ -2590,7 +2675,7 @@
       </c>
       <c r="C41" s="11" t="inlineStr">
         <is>
-          <t>Repeated statements feel more true, even when we know we should check them.</t>
+          <t>The tendency for repeated statements to feel more true, simply because they have become familiar.</t>
         </is>
       </c>
       <c r="D41" s="11" t="inlineStr">
@@ -2616,6 +2701,16 @@
       <c r="H41" s="11" t="n">
         <v>2</v>
       </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Mere Exposure Effect, Confirmation Bias</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Illusory_truth_effect</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="11" t="inlineStr">
@@ -2630,7 +2725,7 @@
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>We explain other people's actions by their character, but our own by the situation.</t>
+          <t>The tendency to explain other people’s behaviour by their character, while explaining our own behaviour by the situation we were in.</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -2656,6 +2751,16 @@
       <c r="H42" s="11" t="n">
         <v>3</v>
       </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Fundamental Attribution Error, Self-serving Bias</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Actor%E2%80%93observer_asymmetry</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="11" t="inlineStr">
@@ -2670,7 +2775,7 @@
       </c>
       <c r="C43" s="11" t="inlineStr">
         <is>
-          <t>We notice biases in others more easily than in ourselves.</t>
+          <t>The tendency to recognise cognitive biases more easily in other people than in ourselves.</t>
         </is>
       </c>
       <c r="D43" s="11" t="inlineStr">
@@ -2696,6 +2801,16 @@
       <c r="H43" s="11" t="n">
         <v>3</v>
       </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Naive Realism, Overconfidence Effect</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Bias_blind_spot</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="11" t="inlineStr">
@@ -2710,7 +2825,7 @@
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>We believe we see reality directly and that reasonable people should agree with us.</t>
+          <t>The belief that we see the world objectively, and that people who disagree with us must be uninformed, irrational, or biased.</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -2736,6 +2851,16 @@
       <c r="H44" s="11" t="n">
         <v>3</v>
       </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>False Consensus Effect, Bias Blind Spot</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Na%C3%AFve_realism_(psychology)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="11" t="inlineStr">
@@ -2750,7 +2875,7 @@
       </c>
       <c r="C45" s="11" t="inlineStr">
         <is>
-          <t>We assume people generally get what they deserve, and search for reasons bad outcomes were earned.</t>
+          <t>The tendency to assume the world is fair and that people usually get what they deserve, which can lead us to blame victims or downplay luck.</t>
         </is>
       </c>
       <c r="D45" s="11" t="inlineStr">
@@ -2776,6 +2901,16 @@
       <c r="H45" s="11" t="n">
         <v>3</v>
       </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Fundamental Attribution Error, Hindsight Bias</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Just-world_hypothesis</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="11" t="inlineStr">
@@ -2790,7 +2925,7 @@
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>We interpret ambiguous actions from others as intentionally hostile or unkind.</t>
+          <t>The tendency to interpret ambiguous actions from others as intentionally hostile, unkind, or personally directed.</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -2816,6 +2951,16 @@
       <c r="H46" s="11" t="n">
         <v>3</v>
       </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Fundamental Attribution Error, Negativity Bias</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Hostile_attribution_bias</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="11" t="inlineStr">
@@ -2830,7 +2975,7 @@
       </c>
       <c r="C47" s="11" t="inlineStr">
         <is>
-          <t>We remember our own role in events as larger and more central than it was.</t>
+          <t>The tendency to remember our own role, effort, or importance in joint events as larger than it really was.</t>
         </is>
       </c>
       <c r="D47" s="11" t="inlineStr">
@@ -2856,6 +3001,16 @@
       <c r="H47" s="11" t="n">
         <v>3</v>
       </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Self-serving Bias, Spotlight Effect</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Egocentric_bias</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="11" t="inlineStr">
@@ -2870,7 +3025,7 @@
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>We overestimate how clearly others can read our emotions and thoughts.</t>
+          <t>The tendency to overestimate how easily other people can read our emotions, thoughts, or internal state.</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
@@ -2896,6 +3051,16 @@
       <c r="H48" s="11" t="n">
         <v>3</v>
       </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Spotlight Effect, Egocentric Bias</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Illusion_of_transparency</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="11" t="inlineStr">
@@ -2910,7 +3075,7 @@
       </c>
       <c r="C49" s="11" t="inlineStr">
         <is>
-          <t>We prefer smaller rewards now over larger rewards later, more steeply than calm planning would suggest.</t>
+          <t>The tendency to prefer smaller rewards now over larger rewards later, more steeply than a calm long-term plan would suggest.</t>
         </is>
       </c>
       <c r="D49" s="11" t="inlineStr">
@@ -2936,6 +3101,16 @@
       <c r="H49" s="11" t="n">
         <v>3</v>
       </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Optimism Bias, Restraint Bias</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Hyperbolic_discounting</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="11" t="inlineStr">
@@ -2950,7 +3125,7 @@
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>We avoid options when the odds of a good outcome are unclear, even if they might be favourable.</t>
+          <t>The tendency to avoid options when the probability of a good outcome is unclear, even if those options could be better than a known alternative.</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -2976,6 +3151,16 @@
       <c r="H50" s="11" t="n">
         <v>3</v>
       </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Status Quo Bias, Loss Aversion</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Ambiguity_effect</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="11" t="inlineStr">
@@ -2990,7 +3175,7 @@
       </c>
       <c r="C51" s="11" t="inlineStr">
         <is>
-          <t>We respond more strongly to one identifiable person in need than to large, statistical groups.</t>
+          <t>The tendency to feel and give more help in response to one identifiable person in need than to large groups described only with statistics.</t>
         </is>
       </c>
       <c r="D51" s="11" t="inlineStr">
@@ -3016,6 +3201,16 @@
       <c r="H51" s="11" t="n">
         <v>3</v>
       </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Availability Heuristic, Negativity Bias</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Identifiable_victim_effect</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="11" t="inlineStr">
@@ -3030,7 +3225,7 @@
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>We overestimate our ability to resist temptation in the moment.</t>
+          <t>The tendency to overestimate how well we will resist temptation when the moment actually arrives.</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
@@ -3056,6 +3251,16 @@
       <c r="H52" s="11" t="n">
         <v>3</v>
       </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Overconfidence Effect, Optimism Bias</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Restraint_bias</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="11" t="inlineStr">
@@ -3070,7 +3275,7 @@
       </c>
       <c r="C53" s="11" t="inlineStr">
         <is>
-          <t>When we feel our freedom is threatened, we push back — sometimes by doing the opposite.</t>
+          <t>The tendency to push back when we feel our freedom is being restricted — sometimes by doing the opposite of what we are urged to do.</t>
         </is>
       </c>
       <c r="D53" s="11" t="inlineStr">
@@ -3096,6 +3301,16 @@
       <c r="H53" s="11" t="n">
         <v>3</v>
       </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Status Quo Bias</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Reactance_(psychology)</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="11" t="inlineStr">
@@ -3110,7 +3325,7 @@
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>We avoid information that might force us to face an uncomfortable problem.</t>
+          <t>The tendency to avoid looking at information that might confirm a problem we would rather not face.</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
@@ -3136,6 +3351,16 @@
       <c r="H54" s="11" t="n">
         <v>3</v>
       </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Optimism Bias, Normalcy Bias</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Ostrich_effect</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="11" t="inlineStr">
@@ -3150,7 +3375,7 @@
       </c>
       <c r="C55" s="11" t="inlineStr">
         <is>
-          <t>We treat situations as if one person's gain must mean another person's loss, even when both could benefit.</t>
+          <t>The tendency to treat a situation as if one person’s gain must mean another person’s loss, even when both could benefit.</t>
         </is>
       </c>
       <c r="D55" s="11" t="inlineStr">
@@ -3176,6 +3401,16 @@
       <c r="H55" s="11" t="n">
         <v>3</v>
       </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>In-group Bias</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Zero-sum_thinking</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="11" t="inlineStr">
@@ -3190,7 +3425,7 @@
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>We judge the morality of an action partly by how lucky or unlucky the outcome was.</t>
+          <t>The tendency to judge how good or bad a decision was partly by how lucky or unlucky the outcome turned out to be.</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
@@ -3216,6 +3451,16 @@
       <c r="H56" s="11" t="n">
         <v>3</v>
       </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Hindsight Bias, Fundamental Attribution Error</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Moral_luck</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="11" t="inlineStr">
@@ -3230,7 +3475,7 @@
       </c>
       <c r="C57" s="11" t="inlineStr">
         <is>
-          <t>We notice a cluster first, then draw a target around it as if we predicted it.</t>
+          <t>The tendency to notice a cluster in data first, then treat that cluster as if it had been predicted — drawing the target after the shots.</t>
         </is>
       </c>
       <c r="D57" s="11" t="inlineStr">
@@ -3256,6 +3501,16 @@
       <c r="H57" s="11" t="n">
         <v>3</v>
       </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Clustering Illusion, Illusory Correlation</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Texas_sharpshooter_fallacy</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="11" t="inlineStr">
@@ -3270,7 +3525,7 @@
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>We are more certain of our judgments than our accuracy usually supports.</t>
+          <t>The tendency to be more confident in our judgments than our actual accuracy usually supports.</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
@@ -3296,6 +3551,16 @@
       <c r="H58" s="11" t="n">
         <v>3</v>
       </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Dunning-Kruger Effect, Optimism Bias</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Overconfidence_effect</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="11" t="inlineStr">
@@ -3310,7 +3575,7 @@
       </c>
       <c r="C59" s="11" t="inlineStr">
         <is>
-          <t>We assume a new tool or change will help more than it does, and overlook its limits.</t>
+          <t>The tendency to assume a new idea, tool, or innovation will help more than it will, while underestimating its limits and side effects.</t>
         </is>
       </c>
       <c r="D59" s="11" t="inlineStr">
@@ -3336,6 +3601,16 @@
       <c r="H59" s="11" t="n">
         <v>3</v>
       </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Optimism Bias, Authority Bias</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Pro-innovation_bias</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="11" t="inlineStr">
@@ -3350,7 +3625,7 @@
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>We reject new evidence or ideas because they challenge established norms or beliefs.</t>
+          <t>The tendency to reject new evidence or ideas mainly because they challenge established beliefs, habits, or authority.</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr">
@@ -3376,6 +3651,16 @@
       <c r="H60" s="11" t="n">
         <v>3</v>
       </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Belief Perseverance, Confirmation Bias</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Semmelweis_reflex</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="11" t="inlineStr">
@@ -3390,7 +3675,7 @@
       </c>
       <c r="C61" s="11" t="inlineStr">
         <is>
-          <t>We take more risks when we feel safer, partly offsetting the protection we gained.</t>
+          <t>The tendency to take greater risks when we feel protected, which can partly cancel out the safety we gained.</t>
         </is>
       </c>
       <c r="D61" s="11" t="inlineStr">
@@ -3415,6 +3700,16 @@
       </c>
       <c r="H61" s="11" t="n">
         <v>3</v>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Optimism Bias, Illusion of Control</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Risk_compensation</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>